<commit_message>
Add customer note and tracking rules
</commit_message>
<xml_diff>
--- a/订单分表模版.xlsx
+++ b/订单分表模版.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>导入编号</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t>客服备注</t>
+  </si>
+  <si>
+    <t>客户备注</t>
   </si>
   <si>
     <t>客户账号</t>
@@ -866,7 +869,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -891,16 +894,10 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -908,9 +905,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1257,135 +1251,129 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultColWidth="10.6296296296296" defaultRowHeight="37" customHeight="1" outlineLevelRow="5"/>
   <cols>
-    <col min="1" max="1" width="22.25" style="17" customWidth="1"/>
-    <col min="2" max="2" width="8.25" style="17" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5" style="17" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="30.7777777777778" style="17" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="32.4444444444444" style="17" customWidth="1"/>
-    <col min="6" max="6" width="10.6296296296296" style="17" customWidth="1"/>
-    <col min="7" max="7" width="10.5" style="17" customWidth="1"/>
-    <col min="8" max="8" width="15" style="17" customWidth="1"/>
-    <col min="9" max="9" width="22" style="17" customWidth="1"/>
-    <col min="10" max="10" width="23.3333333333333" style="17" customWidth="1"/>
-    <col min="11" max="11" width="17.5555555555556" style="17" customWidth="1"/>
-    <col min="12" max="15" width="24.6666666666667" style="17" customWidth="1"/>
-    <col min="16" max="16" width="24.6666666666667" style="18" customWidth="1"/>
-    <col min="17" max="17" width="35.8796296296296" style="17" customWidth="1"/>
-    <col min="18" max="16384" width="10.6296296296296" style="17"/>
+    <col min="1" max="1" width="22.25" style="14" customWidth="1"/>
+    <col min="2" max="2" width="8.25" style="14" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5" style="14" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="30.7777777777778" style="14" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="32.4444444444444" style="14" customWidth="1"/>
+    <col min="6" max="6" width="10.6296296296296" style="14" customWidth="1"/>
+    <col min="7" max="7" width="10.5" style="14" customWidth="1"/>
+    <col min="8" max="9" width="15" style="14" customWidth="1"/>
+    <col min="10" max="10" width="22" style="14" customWidth="1"/>
+    <col min="11" max="11" width="23.3333333333333" style="14" customWidth="1"/>
+    <col min="12" max="12" width="17.5555555555556" style="14" customWidth="1"/>
+    <col min="13" max="16" width="24.6666666666667" style="14" customWidth="1"/>
+    <col min="17" max="17" width="24.6666666666667" style="15" customWidth="1"/>
+    <col min="18" max="18" width="35.8796296296296" style="14" customWidth="1"/>
+    <col min="19" max="16384" width="10.6296296296296" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" s="16" customFormat="1" customHeight="1" spans="1:16">
-      <c r="A1" s="16" t="s">
+    <row r="1" s="13" customFormat="1" customHeight="1" spans="1:17">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="J1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:17">
-      <c r="A2" s="19"/>
-      <c r="E2" s="20"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="22" t="s">
+      <c r="Q1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="17" t="s">
+    </row>
+    <row r="2" customHeight="1" spans="1:18">
+      <c r="A2" s="16"/>
+      <c r="E2" s="17"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="M2" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="24"/>
-    </row>
-    <row r="3" customHeight="1" spans="5:16">
-      <c r="E3" s="21"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="P3" s="23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="8:16">
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="P4" s="23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" spans="9:16">
-      <c r="I5" s="22"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="P5" s="23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" customHeight="1" spans="8:16">
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="P6" s="23" t="s">
-        <v>20</v>
+      <c r="Q2" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="R2" s="21"/>
+    </row>
+    <row r="3" customHeight="1" spans="5:17">
+      <c r="E3" s="18"/>
+      <c r="J3" s="19"/>
+      <c r="Q3" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="8:17">
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="Q4" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="10:17">
+      <c r="J5" s="19"/>
+      <c r="Q5" s="20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="8:17">
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="Q6" s="20" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1413,46 +1401,46 @@
   <sheetData>
     <row r="1" ht="15.6" spans="1:7">
       <c r="A1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="4"/>
       <c r="B2" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1494,64 +1482,64 @@
       <c r="C7" s="7"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
     </row>
     <row r="8" spans="2:7">
       <c r="B8" s="5"/>
       <c r="C8" s="7"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
     </row>
     <row r="9" spans="2:7">
       <c r="B9" s="5"/>
       <c r="C9" s="7"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
     </row>
     <row r="10" spans="2:7">
       <c r="B10" s="5"/>
       <c r="C10" s="7"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
     </row>
     <row r="11" spans="2:7">
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
     </row>
     <row r="12" spans="2:7">
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
     </row>
     <row r="13" spans="2:7">
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="2:7">
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" s="1" customFormat="1" spans="1:7">
       <c r="A15" s="4"/>
@@ -1564,68 +1552,68 @@
     </row>
     <row r="16" s="1" customFormat="1" spans="1:7">
       <c r="A16" s="4"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="2:7">
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="14"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="12"/>
     </row>
     <row r="18" spans="2:7">
-      <c r="B18" s="14"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="14"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="12"/>
     </row>
     <row r="19" spans="2:7">
-      <c r="B19" s="14"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="14"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="12"/>
     </row>
     <row r="20" spans="2:7">
-      <c r="B20" s="14"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="14"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="12"/>
     </row>
     <row r="21" spans="2:7">
-      <c r="B21" s="14"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="14"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="12"/>
     </row>
     <row r="22" spans="2:7">
-      <c r="B22" s="12"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="14"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="12"/>
     </row>
     <row r="23" spans="2:7">
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>